<commit_message>
Add Fast Track PDF report pipeline with reliable Excel recalc and bot auto-workbook resolution.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backend/templates/fdd/CF_NA_L3_order.xlsx
+++ b/backend/templates/fdd/CF_NA_L3_order.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="L3_order" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,21 +413,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>L3</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -568,12 +556,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>DL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cash &amp; cash equivalents</t>
+          <t>Financial liabilities</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -592,7 +580,112 @@
         </is>
       </c>
       <c r="C11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Subscribed capital</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Capital surplus</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Retained earnings</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Retained profits</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Net retained profits</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Net profit</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Profit distribution</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>